<commit_message>
Lead-Tracker: alle Farben auf Schwarz-Weiß umgestellt
Basis ist die von Kevin neu hochgeladene Lead-Tracker.xlsx (14 Spalten,
leere Beispieltabelle). Alle Akzentfarben ersetzt durch Schwarz (#111111)
und Weiß (#ffffff): Kopfzeilen-Fill (vorher Blau), Eingabezellen-Schrift
(vorher Blau) und Formel-Schrift jetzt einheitlich Schwarz. Die
Prioritäts-Markierung (Spalte Priorität, A/B/C) ließ sich mit nur zwei
Farben nicht mehr dreistufig farblich unterscheiden, deshalb hebt jetzt nur
noch "A" farblich hervor (schwarze Füllung, weiße Schrift), "B" und "C"
bleiben ungefärbt. Den Hinweistext in der Anleitung, der sich auf "blaue
Schrift" bezog, entsprechend umformuliert.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DeqSdBatYE6t9FA6GS9TPf
</commit_message>
<xml_diff>
--- a/vertrieb/Lead-Tracker.xlsx
+++ b/vertrieb/Lead-Tracker.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="57">
   <si>
     <t xml:space="preserve">Lead-Scoring-System – Recognize You</t>
   </si>
@@ -128,7 +128,7 @@
     <t xml:space="preserve">- eigene Sichtprüfung der Website: Design, Mobilansicht, Ladezeit, Aktualität</t>
   </si>
   <si>
-    <t xml:space="preserve">Nur die Zellen mit blauer Schrift im Lead-Tracker ausfüllen. Gesamtscore und Priorität berechnen sich automatisch.</t>
+    <t xml:space="preserve">Nur die Spalten Website-Schwäche, Unternehmensgröße, Entscheider erreichbar und Problembewusstsein im Lead-Tracker ausfüllen. Gesamtscore und Priorität berechnen sich automatisch.</t>
   </si>
   <si>
     <t xml:space="preserve">Firma</t>
@@ -167,6 +167,9 @@
     <t xml:space="preserve">Status</t>
   </si>
   <si>
+    <t xml:space="preserve">Nächster Schritt / Termin</t>
+  </si>
+  <si>
     <t xml:space="preserve">Notizen</t>
   </si>
   <si>
@@ -189,149 +192,16 @@
   </si>
   <si>
     <t xml:space="preserve">Beispielzeile, kann überschrieben werden.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gollitscher Bau GmbH &amp; Co. KG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bauunternehmen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gollitscher-bau.de</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Erich Gollitscher</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09172 4789957 / info@gollitscher-bau.de</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adresse: Lorenzberg 15, 91166 Georgensgmünd. Erich Gollitscher ist laut Handelsregister (North Data) Geschaeftsfuehrer der Gollitscher Verwaltungs GmbH, der persoenlich haftenden Gesellschafterin. Website vorhanden, Qualitaet manuell pruefen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R&amp;M Versorgungstechnik GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Heizung, Sanitaer, Klima, Elektro, Solar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rm-versorgungstechnik.de</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ralf Menzel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09172 685470</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adresse: Breitenloher Weg 15, 91166 Georgensgmünd. Ralf Menzel laut Handelsregister (North Data) Geschaeftsfuehrer, zweiter Geschaeftsfuehrer Rainer Mory. Website vorhanden, Qualitaet manuell pruefen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wenzel Heizungs- und Sanitaertechnik GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Heizung, Sanitaer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wenzel-heizung.de</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bernd Herzog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09172 6953-0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adresse: Breitenloher Weg 19, 91166 Georgensgmünd. Bernd Herzog laut Handelsregister (North Data) Geschaeftsfuehrer. Gegruendet 1897. Website vorhanden, Qualitaet manuell pruefen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Autoservice Georgensgmünd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KFZ-Werkstatt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">autoservice-georgensgmuend.de</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stefan Buckl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adresse: Pleinfelder Str. 72, 91166 Georgensgmünd. Stefan Buckl laut Unternehmensbeschreibung Inhaber. Website vorhanden, Qualitaet manuell pruefen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Steuerkanzlei Thorsten Alt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Steuerberatung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">steuerkanzlei-alt.de</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thorsten Alt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09172 4850730</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adresse: Pleinfelder Strasse 34, 91166 Georgensgmünd. Thorsten Alt ist der namensgebende Steuerberater und Kanzleiinhaber. Website vorhanden, Qualitaet manuell pruefen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meromi Frisoergeschaefte GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Friseur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">keine eigene Website gefunden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peter Fexer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adresse: Egid-Harrer-Str. 72, 91166 Georgensgmünd. Peter Fexer laut Handelsregister (North Data) Geschaeftsfuehrer, Unternehmen betreibt laut Registereintrag 4 Standorte.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gsänger Bau-GmbH (Gsänger Bauunternehmung)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bauunternehmen, Hoch- und Tiefbau</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jochen Schraff</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09172 6951-0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adresse: An der Papiermühle 43, 91166 Georgensgmünd. Jochen Schraff laut Handelsregister (North Data) Geschaeftsfuehrer, sitzt laut Eintrag in Augsburg, Gesellschafter ist TSG Deutschland GmbH &amp; Co. KG. Moeglicherweise Teil eines groesseren Konzerns, vor Anruf pruefen ob das noch zur Zielgruppe passt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Emil Kiessling GmbH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hersteller chemisch-pharmazeutischer/kosmetischer Produkte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nicht recherchiert</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Martina Reichardt-Demirtas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Martina Reichardt-Demirtas laut Handelsregister (North Data) Geschaeftsfuehrerin. Groesserer, etablierter Hersteller vor Ort, moeglicherweise schon professionelle Website und zu gross fuer die Zielgruppe, vor Anruf pruefen.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="General"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -357,7 +227,7 @@
     <font>
       <b val="true"/>
       <sz val="16"/>
-      <color rgb="FF1F4E78"/>
+      <color rgb="FF111111"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -371,7 +241,7 @@
     <font>
       <b val="true"/>
       <sz val="12"/>
-      <color rgb="FF1F4E78"/>
+      <color rgb="FF111111"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -393,14 +263,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color rgb="FF111111"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -415,8 +278,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E78"/>
-        <bgColor rgb="FF003366"/>
+        <fgColor rgb="FF111111"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -474,7 +337,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -482,7 +349,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -494,15 +361,15 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -514,12 +381,8 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -539,25 +402,24 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
+      <font>
+        <color rgb="FFFFFFFF"/>
+      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FF111111"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF111111"/>
+      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFFFFF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -598,12 +460,12 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFC6EFCE"/>
-      <rgbColor rgb="FFFFEB9C"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFC7CE"/>
+      <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -614,11 +476,11 @@
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF111111"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF1F4E78"/>
+      <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
     </indexedColors>
   </colors>
@@ -808,185 +670,185 @@
   <dimension ref="A1:C26"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="70"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="7" t="s">
+      <c r="C16" s="8" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="8" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="s">
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="8" t="s">
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8" t="s">
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="s">
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1014,1028 +876,966 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="6" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="6" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="5" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="5" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="F2" s="10" t="n">
+      <c r="E2" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F2" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="G2" s="10" t="n">
+      <c r="G2" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="H2" s="10" t="n">
+      <c r="H2" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="I2" s="10" t="n">
+      <c r="I2" s="11" t="n">
         <v>1</v>
       </c>
       <c r="J2" s="11" t="n">
         <f aca="false">IF(COUNT(F2:I2)=0,"",SUM(F2:I2))</f>
         <v>8</v>
       </c>
-      <c r="K2" s="12" t="str">
+      <c r="K2" s="11" t="str">
         <f aca="false">IF(J2="","",IF(J2&gt;=8,"A",IF(J2&gt;=5,"B","C")))</f>
         <v>A</v>
       </c>
-      <c r="L2" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="M2" s="13" t="s">
+      <c r="L2" s="8" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
+      <c r="M2" s="12"/>
+      <c r="N2" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="E3" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
       <c r="J3" s="11" t="str">
         <f aca="false">IF(COUNT(F3:I3)=0,"",SUM(F3:I3))</f>
         <v/>
       </c>
-      <c r="K3" s="12" t="str">
+      <c r="K3" s="11" t="str">
         <f aca="false">IF(J3="","",IF(J3&gt;=8,"A",IF(J3&gt;=5,"B","C")))</f>
         <v/>
       </c>
-      <c r="L3" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="M3" s="14" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
+      <c r="N3" s="14"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
       <c r="J4" s="11" t="str">
         <f aca="false">IF(COUNT(F4:I4)=0,"",SUM(F4:I4))</f>
         <v/>
       </c>
-      <c r="K4" s="12" t="str">
+      <c r="K4" s="11" t="str">
         <f aca="false">IF(J4="","",IF(J4&gt;=8,"A",IF(J4&gt;=5,"B","C")))</f>
         <v/>
       </c>
-      <c r="L4" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="M4" s="14" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
+      <c r="L4" s="14"/>
+      <c r="M4" s="14"/>
+      <c r="N4" s="14"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
       <c r="J5" s="11" t="str">
         <f aca="false">IF(COUNT(F5:I5)=0,"",SUM(F5:I5))</f>
         <v/>
       </c>
-      <c r="K5" s="12" t="str">
+      <c r="K5" s="11" t="str">
         <f aca="false">IF(J5="","",IF(J5&gt;=8,"A",IF(J5&gt;=5,"B","C")))</f>
         <v/>
       </c>
-      <c r="L5" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="M5" s="14" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>77</v>
-      </c>
+      <c r="L5" s="14"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="14"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
       <c r="E6" s="14"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
       <c r="J6" s="11" t="str">
         <f aca="false">IF(COUNT(F6:I6)=0,"",SUM(F6:I6))</f>
         <v/>
       </c>
-      <c r="K6" s="12" t="str">
+      <c r="K6" s="11" t="str">
         <f aca="false">IF(J6="","",IF(J6&gt;=8,"A",IF(J6&gt;=5,"B","C")))</f>
         <v/>
       </c>
-      <c r="L6" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="M6" s="14" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
+      <c r="L6" s="14"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="14"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
       <c r="J7" s="11" t="str">
         <f aca="false">IF(COUNT(F7:I7)=0,"",SUM(F7:I7))</f>
         <v/>
       </c>
-      <c r="K7" s="12" t="str">
+      <c r="K7" s="11" t="str">
         <f aca="false">IF(J7="","",IF(J7&gt;=8,"A",IF(J7&gt;=5,"B","C")))</f>
         <v/>
       </c>
-      <c r="L7" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="M7" s="14" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="D8" s="14" t="s">
-        <v>88</v>
-      </c>
+      <c r="L7" s="14"/>
+      <c r="M7" s="14"/>
+      <c r="N7" s="14"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
       <c r="E8" s="14"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
       <c r="J8" s="11" t="str">
         <f aca="false">IF(COUNT(F8:I8)=0,"",SUM(F8:I8))</f>
         <v/>
       </c>
-      <c r="K8" s="12" t="str">
+      <c r="K8" s="11" t="str">
         <f aca="false">IF(J8="","",IF(J8&gt;=8,"A",IF(J8&gt;=5,"B","C")))</f>
         <v/>
       </c>
-      <c r="L8" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="M8" s="14" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="E9" s="14" t="s">
-        <v>93</v>
-      </c>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
+      <c r="L8" s="14"/>
+      <c r="M8" s="14"/>
+      <c r="N8" s="14"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14"/>
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
       <c r="J9" s="11" t="str">
         <f aca="false">IF(COUNT(F9:I9)=0,"",SUM(F9:I9))</f>
         <v/>
       </c>
-      <c r="K9" s="12" t="str">
+      <c r="K9" s="11" t="str">
         <f aca="false">IF(J9="","",IF(J9&gt;=8,"A",IF(J9&gt;=5,"B","C")))</f>
         <v/>
       </c>
-      <c r="L9" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="M9" s="14" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>98</v>
-      </c>
+      <c r="L9" s="14"/>
+      <c r="M9" s="14"/>
+      <c r="N9" s="14"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
       <c r="E10" s="14"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
       <c r="J10" s="11" t="str">
         <f aca="false">IF(COUNT(F10:I10)=0,"",SUM(F10:I10))</f>
         <v/>
       </c>
-      <c r="K10" s="12" t="str">
+      <c r="K10" s="11" t="str">
         <f aca="false">IF(J10="","",IF(J10&gt;=8,"A",IF(J10&gt;=5,"B","C")))</f>
         <v/>
       </c>
-      <c r="L10" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="M10" s="14" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L10" s="14"/>
+      <c r="M10" s="14"/>
+      <c r="N10" s="14"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14"/>
       <c r="B11" s="14"/>
       <c r="C11" s="14"/>
       <c r="D11" s="14"/>
       <c r="E11" s="14"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
       <c r="J11" s="11" t="str">
         <f aca="false">IF(COUNT(F11:I11)=0,"",SUM(F11:I11))</f>
         <v/>
       </c>
-      <c r="K11" s="12" t="str">
+      <c r="K11" s="11" t="str">
         <f aca="false">IF(J11="","",IF(J11&gt;=8,"A",IF(J11&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L11" s="14"/>
       <c r="M11" s="14"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N11" s="14"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14"/>
       <c r="B12" s="14"/>
       <c r="C12" s="14"/>
       <c r="D12" s="14"/>
       <c r="E12" s="14"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="10"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
       <c r="J12" s="11" t="str">
         <f aca="false">IF(COUNT(F12:I12)=0,"",SUM(F12:I12))</f>
         <v/>
       </c>
-      <c r="K12" s="12" t="str">
+      <c r="K12" s="11" t="str">
         <f aca="false">IF(J12="","",IF(J12&gt;=8,"A",IF(J12&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L12" s="14"/>
       <c r="M12" s="14"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N12" s="14"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="14"/>
       <c r="B13" s="14"/>
       <c r="C13" s="14"/>
       <c r="D13" s="14"/>
       <c r="E13" s="14"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
       <c r="J13" s="11" t="str">
         <f aca="false">IF(COUNT(F13:I13)=0,"",SUM(F13:I13))</f>
         <v/>
       </c>
-      <c r="K13" s="12" t="str">
+      <c r="K13" s="11" t="str">
         <f aca="false">IF(J13="","",IF(J13&gt;=8,"A",IF(J13&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L13" s="14"/>
       <c r="M13" s="14"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N13" s="14"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="14"/>
       <c r="D14" s="14"/>
       <c r="E14" s="14"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
       <c r="J14" s="11" t="str">
         <f aca="false">IF(COUNT(F14:I14)=0,"",SUM(F14:I14))</f>
         <v/>
       </c>
-      <c r="K14" s="12" t="str">
+      <c r="K14" s="11" t="str">
         <f aca="false">IF(J14="","",IF(J14&gt;=8,"A",IF(J14&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L14" s="14"/>
       <c r="M14" s="14"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N14" s="14"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="14"/>
       <c r="B15" s="14"/>
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
       <c r="E15" s="14"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
       <c r="J15" s="11" t="str">
         <f aca="false">IF(COUNT(F15:I15)=0,"",SUM(F15:I15))</f>
         <v/>
       </c>
-      <c r="K15" s="12" t="str">
+      <c r="K15" s="11" t="str">
         <f aca="false">IF(J15="","",IF(J15&gt;=8,"A",IF(J15&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L15" s="14"/>
       <c r="M15" s="14"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N15" s="14"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14"/>
       <c r="B16" s="14"/>
       <c r="C16" s="14"/>
       <c r="D16" s="14"/>
       <c r="E16" s="14"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="10"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
       <c r="J16" s="11" t="str">
         <f aca="false">IF(COUNT(F16:I16)=0,"",SUM(F16:I16))</f>
         <v/>
       </c>
-      <c r="K16" s="12" t="str">
+      <c r="K16" s="11" t="str">
         <f aca="false">IF(J16="","",IF(J16&gt;=8,"A",IF(J16&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L16" s="14"/>
       <c r="M16" s="14"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N16" s="14"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="14"/>
       <c r="B17" s="14"/>
       <c r="C17" s="14"/>
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
       <c r="J17" s="11" t="str">
         <f aca="false">IF(COUNT(F17:I17)=0,"",SUM(F17:I17))</f>
         <v/>
       </c>
-      <c r="K17" s="12" t="str">
+      <c r="K17" s="11" t="str">
         <f aca="false">IF(J17="","",IF(J17&gt;=8,"A",IF(J17&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L17" s="14"/>
       <c r="M17" s="14"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N17" s="14"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14"/>
       <c r="B18" s="14"/>
       <c r="C18" s="14"/>
       <c r="D18" s="14"/>
       <c r="E18" s="14"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
       <c r="J18" s="11" t="str">
         <f aca="false">IF(COUNT(F18:I18)=0,"",SUM(F18:I18))</f>
         <v/>
       </c>
-      <c r="K18" s="12" t="str">
+      <c r="K18" s="11" t="str">
         <f aca="false">IF(J18="","",IF(J18&gt;=8,"A",IF(J18&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L18" s="14"/>
       <c r="M18" s="14"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N18" s="14"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="14"/>
       <c r="D19" s="14"/>
       <c r="E19" s="14"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
       <c r="J19" s="11" t="str">
         <f aca="false">IF(COUNT(F19:I19)=0,"",SUM(F19:I19))</f>
         <v/>
       </c>
-      <c r="K19" s="12" t="str">
+      <c r="K19" s="11" t="str">
         <f aca="false">IF(J19="","",IF(J19&gt;=8,"A",IF(J19&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L19" s="14"/>
       <c r="M19" s="14"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N19" s="14"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14"/>
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
       <c r="D20" s="14"/>
       <c r="E20" s="14"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
       <c r="J20" s="11" t="str">
         <f aca="false">IF(COUNT(F20:I20)=0,"",SUM(F20:I20))</f>
         <v/>
       </c>
-      <c r="K20" s="12" t="str">
+      <c r="K20" s="11" t="str">
         <f aca="false">IF(J20="","",IF(J20&gt;=8,"A",IF(J20&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L20" s="14"/>
       <c r="M20" s="14"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N20" s="14"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="14"/>
       <c r="B21" s="14"/>
       <c r="C21" s="14"/>
       <c r="D21" s="14"/>
       <c r="E21" s="14"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="10"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
       <c r="J21" s="11" t="str">
         <f aca="false">IF(COUNT(F21:I21)=0,"",SUM(F21:I21))</f>
         <v/>
       </c>
-      <c r="K21" s="12" t="str">
+      <c r="K21" s="11" t="str">
         <f aca="false">IF(J21="","",IF(J21&gt;=8,"A",IF(J21&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L21" s="14"/>
       <c r="M21" s="14"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N21" s="14"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="14"/>
       <c r="B22" s="14"/>
       <c r="C22" s="14"/>
       <c r="D22" s="14"/>
       <c r="E22" s="14"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="10"/>
-      <c r="I22" s="10"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
       <c r="J22" s="11" t="str">
         <f aca="false">IF(COUNT(F22:I22)=0,"",SUM(F22:I22))</f>
         <v/>
       </c>
-      <c r="K22" s="12" t="str">
+      <c r="K22" s="11" t="str">
         <f aca="false">IF(J22="","",IF(J22&gt;=8,"A",IF(J22&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L22" s="14"/>
       <c r="M22" s="14"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N22" s="14"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="14"/>
       <c r="B23" s="14"/>
       <c r="C23" s="14"/>
       <c r="D23" s="14"/>
       <c r="E23" s="14"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="10"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
       <c r="J23" s="11" t="str">
         <f aca="false">IF(COUNT(F23:I23)=0,"",SUM(F23:I23))</f>
         <v/>
       </c>
-      <c r="K23" s="12" t="str">
+      <c r="K23" s="11" t="str">
         <f aca="false">IF(J23="","",IF(J23&gt;=8,"A",IF(J23&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L23" s="14"/>
       <c r="M23" s="14"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N23" s="14"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="14"/>
       <c r="B24" s="14"/>
       <c r="C24" s="14"/>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="10"/>
-      <c r="I24" s="10"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
       <c r="J24" s="11" t="str">
         <f aca="false">IF(COUNT(F24:I24)=0,"",SUM(F24:I24))</f>
         <v/>
       </c>
-      <c r="K24" s="12" t="str">
+      <c r="K24" s="11" t="str">
         <f aca="false">IF(J24="","",IF(J24&gt;=8,"A",IF(J24&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L24" s="14"/>
       <c r="M24" s="14"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N24" s="14"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="14"/>
       <c r="B25" s="14"/>
       <c r="C25" s="14"/>
       <c r="D25" s="14"/>
       <c r="E25" s="14"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="10"/>
-      <c r="H25" s="10"/>
-      <c r="I25" s="10"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
       <c r="J25" s="11" t="str">
         <f aca="false">IF(COUNT(F25:I25)=0,"",SUM(F25:I25))</f>
         <v/>
       </c>
-      <c r="K25" s="12" t="str">
+      <c r="K25" s="11" t="str">
         <f aca="false">IF(J25="","",IF(J25&gt;=8,"A",IF(J25&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L25" s="14"/>
       <c r="M25" s="14"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N25" s="14"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="14"/>
       <c r="B26" s="14"/>
       <c r="C26" s="14"/>
       <c r="D26" s="14"/>
       <c r="E26" s="14"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
-      <c r="H26" s="10"/>
-      <c r="I26" s="10"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="11"/>
       <c r="J26" s="11" t="str">
         <f aca="false">IF(COUNT(F26:I26)=0,"",SUM(F26:I26))</f>
         <v/>
       </c>
-      <c r="K26" s="12" t="str">
+      <c r="K26" s="11" t="str">
         <f aca="false">IF(J26="","",IF(J26&gt;=8,"A",IF(J26&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L26" s="14"/>
       <c r="M26" s="14"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N26" s="14"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="14"/>
       <c r="B27" s="14"/>
       <c r="C27" s="14"/>
       <c r="D27" s="14"/>
       <c r="E27" s="14"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
-      <c r="H27" s="10"/>
-      <c r="I27" s="10"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
       <c r="J27" s="11" t="str">
         <f aca="false">IF(COUNT(F27:I27)=0,"",SUM(F27:I27))</f>
         <v/>
       </c>
-      <c r="K27" s="12" t="str">
+      <c r="K27" s="11" t="str">
         <f aca="false">IF(J27="","",IF(J27&gt;=8,"A",IF(J27&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L27" s="14"/>
       <c r="M27" s="14"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N27" s="14"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="14"/>
       <c r="B28" s="14"/>
       <c r="C28" s="14"/>
       <c r="D28" s="14"/>
       <c r="E28" s="14"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="10"/>
-      <c r="H28" s="10"/>
-      <c r="I28" s="10"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="11"/>
       <c r="J28" s="11" t="str">
         <f aca="false">IF(COUNT(F28:I28)=0,"",SUM(F28:I28))</f>
         <v/>
       </c>
-      <c r="K28" s="12" t="str">
+      <c r="K28" s="11" t="str">
         <f aca="false">IF(J28="","",IF(J28&gt;=8,"A",IF(J28&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L28" s="14"/>
       <c r="M28" s="14"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N28" s="14"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="14"/>
       <c r="B29" s="14"/>
       <c r="C29" s="14"/>
       <c r="D29" s="14"/>
       <c r="E29" s="14"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="10"/>
-      <c r="H29" s="10"/>
-      <c r="I29" s="10"/>
+      <c r="F29" s="11"/>
+      <c r="G29" s="11"/>
+      <c r="H29" s="11"/>
+      <c r="I29" s="11"/>
       <c r="J29" s="11" t="str">
         <f aca="false">IF(COUNT(F29:I29)=0,"",SUM(F29:I29))</f>
         <v/>
       </c>
-      <c r="K29" s="12" t="str">
+      <c r="K29" s="11" t="str">
         <f aca="false">IF(J29="","",IF(J29&gt;=8,"A",IF(J29&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L29" s="14"/>
       <c r="M29" s="14"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N29" s="14"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="14"/>
       <c r="B30" s="14"/>
       <c r="C30" s="14"/>
       <c r="D30" s="14"/>
       <c r="E30" s="14"/>
-      <c r="F30" s="10"/>
-      <c r="G30" s="10"/>
-      <c r="H30" s="10"/>
-      <c r="I30" s="10"/>
+      <c r="F30" s="11"/>
+      <c r="G30" s="11"/>
+      <c r="H30" s="11"/>
+      <c r="I30" s="11"/>
       <c r="J30" s="11" t="str">
         <f aca="false">IF(COUNT(F30:I30)=0,"",SUM(F30:I30))</f>
         <v/>
       </c>
-      <c r="K30" s="12" t="str">
+      <c r="K30" s="11" t="str">
         <f aca="false">IF(J30="","",IF(J30&gt;=8,"A",IF(J30&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L30" s="14"/>
       <c r="M30" s="14"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N30" s="14"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="14"/>
       <c r="B31" s="14"/>
       <c r="C31" s="14"/>
       <c r="D31" s="14"/>
       <c r="E31" s="14"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="10"/>
-      <c r="H31" s="10"/>
-      <c r="I31" s="10"/>
+      <c r="F31" s="11"/>
+      <c r="G31" s="11"/>
+      <c r="H31" s="11"/>
+      <c r="I31" s="11"/>
       <c r="J31" s="11" t="str">
         <f aca="false">IF(COUNT(F31:I31)=0,"",SUM(F31:I31))</f>
         <v/>
       </c>
-      <c r="K31" s="12" t="str">
+      <c r="K31" s="11" t="str">
         <f aca="false">IF(J31="","",IF(J31&gt;=8,"A",IF(J31&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L31" s="14"/>
       <c r="M31" s="14"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N31" s="14"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="14"/>
       <c r="B32" s="14"/>
       <c r="C32" s="14"/>
       <c r="D32" s="14"/>
       <c r="E32" s="14"/>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10"/>
-      <c r="H32" s="10"/>
-      <c r="I32" s="10"/>
+      <c r="F32" s="11"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="11"/>
+      <c r="I32" s="11"/>
       <c r="J32" s="11" t="str">
         <f aca="false">IF(COUNT(F32:I32)=0,"",SUM(F32:I32))</f>
         <v/>
       </c>
-      <c r="K32" s="12" t="str">
+      <c r="K32" s="11" t="str">
         <f aca="false">IF(J32="","",IF(J32&gt;=8,"A",IF(J32&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L32" s="14"/>
       <c r="M32" s="14"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N32" s="14"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="14"/>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
       <c r="D33" s="14"/>
       <c r="E33" s="14"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="10"/>
-      <c r="H33" s="10"/>
-      <c r="I33" s="10"/>
+      <c r="F33" s="11"/>
+      <c r="G33" s="11"/>
+      <c r="H33" s="11"/>
+      <c r="I33" s="11"/>
       <c r="J33" s="11" t="str">
         <f aca="false">IF(COUNT(F33:I33)=0,"",SUM(F33:I33))</f>
         <v/>
       </c>
-      <c r="K33" s="12" t="str">
+      <c r="K33" s="11" t="str">
         <f aca="false">IF(J33="","",IF(J33&gt;=8,"A",IF(J33&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L33" s="14"/>
       <c r="M33" s="14"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N33" s="14"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="14"/>
       <c r="B34" s="14"/>
       <c r="C34" s="14"/>
       <c r="D34" s="14"/>
       <c r="E34" s="14"/>
-      <c r="F34" s="10"/>
-      <c r="G34" s="10"/>
-      <c r="H34" s="10"/>
-      <c r="I34" s="10"/>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="11"/>
+      <c r="I34" s="11"/>
       <c r="J34" s="11" t="str">
         <f aca="false">IF(COUNT(F34:I34)=0,"",SUM(F34:I34))</f>
         <v/>
       </c>
-      <c r="K34" s="12" t="str">
+      <c r="K34" s="11" t="str">
         <f aca="false">IF(J34="","",IF(J34&gt;=8,"A",IF(J34&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L34" s="14"/>
       <c r="M34" s="14"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N34" s="14"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="14"/>
       <c r="B35" s="14"/>
       <c r="C35" s="14"/>
       <c r="D35" s="14"/>
       <c r="E35" s="14"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
-      <c r="I35" s="10"/>
+      <c r="F35" s="11"/>
+      <c r="G35" s="11"/>
+      <c r="H35" s="11"/>
+      <c r="I35" s="11"/>
       <c r="J35" s="11" t="str">
         <f aca="false">IF(COUNT(F35:I35)=0,"",SUM(F35:I35))</f>
         <v/>
       </c>
-      <c r="K35" s="12" t="str">
+      <c r="K35" s="11" t="str">
         <f aca="false">IF(J35="","",IF(J35&gt;=8,"A",IF(J35&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L35" s="14"/>
       <c r="M35" s="14"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N35" s="14"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="14"/>
       <c r="B36" s="14"/>
       <c r="C36" s="14"/>
       <c r="D36" s="14"/>
       <c r="E36" s="14"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="10"/>
-      <c r="I36" s="10"/>
+      <c r="F36" s="11"/>
+      <c r="G36" s="11"/>
+      <c r="H36" s="11"/>
+      <c r="I36" s="11"/>
       <c r="J36" s="11" t="str">
         <f aca="false">IF(COUNT(F36:I36)=0,"",SUM(F36:I36))</f>
         <v/>
       </c>
-      <c r="K36" s="12" t="str">
+      <c r="K36" s="11" t="str">
         <f aca="false">IF(J36="","",IF(J36&gt;=8,"A",IF(J36&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L36" s="14"/>
       <c r="M36" s="14"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N36" s="14"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="14"/>
       <c r="B37" s="14"/>
       <c r="C37" s="14"/>
       <c r="D37" s="14"/>
       <c r="E37" s="14"/>
-      <c r="F37" s="10"/>
-      <c r="G37" s="10"/>
-      <c r="H37" s="10"/>
-      <c r="I37" s="10"/>
+      <c r="F37" s="11"/>
+      <c r="G37" s="11"/>
+      <c r="H37" s="11"/>
+      <c r="I37" s="11"/>
       <c r="J37" s="11" t="str">
         <f aca="false">IF(COUNT(F37:I37)=0,"",SUM(F37:I37))</f>
         <v/>
       </c>
-      <c r="K37" s="12" t="str">
+      <c r="K37" s="11" t="str">
         <f aca="false">IF(J37="","",IF(J37&gt;=8,"A",IF(J37&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L37" s="14"/>
       <c r="M37" s="14"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N37" s="14"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="14"/>
       <c r="B38" s="14"/>
       <c r="C38" s="14"/>
       <c r="D38" s="14"/>
       <c r="E38" s="14"/>
-      <c r="F38" s="10"/>
-      <c r="G38" s="10"/>
-      <c r="H38" s="10"/>
-      <c r="I38" s="10"/>
+      <c r="F38" s="11"/>
+      <c r="G38" s="11"/>
+      <c r="H38" s="11"/>
+      <c r="I38" s="11"/>
       <c r="J38" s="11" t="str">
         <f aca="false">IF(COUNT(F38:I38)=0,"",SUM(F38:I38))</f>
         <v/>
       </c>
-      <c r="K38" s="12" t="str">
+      <c r="K38" s="11" t="str">
         <f aca="false">IF(J38="","",IF(J38&gt;=8,"A",IF(J38&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L38" s="14"/>
       <c r="M38" s="14"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N38" s="14"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="14"/>
       <c r="B39" s="14"/>
       <c r="C39" s="14"/>
       <c r="D39" s="14"/>
       <c r="E39" s="14"/>
-      <c r="F39" s="10"/>
-      <c r="G39" s="10"/>
-      <c r="H39" s="10"/>
-      <c r="I39" s="10"/>
+      <c r="F39" s="11"/>
+      <c r="G39" s="11"/>
+      <c r="H39" s="11"/>
+      <c r="I39" s="11"/>
       <c r="J39" s="11" t="str">
         <f aca="false">IF(COUNT(F39:I39)=0,"",SUM(F39:I39))</f>
         <v/>
       </c>
-      <c r="K39" s="12" t="str">
+      <c r="K39" s="11" t="str">
         <f aca="false">IF(J39="","",IF(J39&gt;=8,"A",IF(J39&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L39" s="14"/>
       <c r="M39" s="14"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N39" s="14"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="14"/>
       <c r="B40" s="14"/>
       <c r="C40" s="14"/>
       <c r="D40" s="14"/>
       <c r="E40" s="14"/>
-      <c r="F40" s="10"/>
-      <c r="G40" s="10"/>
-      <c r="H40" s="10"/>
-      <c r="I40" s="10"/>
+      <c r="F40" s="11"/>
+      <c r="G40" s="11"/>
+      <c r="H40" s="11"/>
+      <c r="I40" s="11"/>
       <c r="J40" s="11" t="str">
         <f aca="false">IF(COUNT(F40:I40)=0,"",SUM(F40:I40))</f>
         <v/>
       </c>
-      <c r="K40" s="12" t="str">
+      <c r="K40" s="11" t="str">
         <f aca="false">IF(J40="","",IF(J40&gt;=8,"A",IF(J40&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L40" s="14"/>
       <c r="M40" s="14"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N40" s="14"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="14"/>
       <c r="B41" s="14"/>
       <c r="C41" s="14"/>
       <c r="D41" s="14"/>
       <c r="E41" s="14"/>
-      <c r="F41" s="10"/>
-      <c r="G41" s="10"/>
-      <c r="H41" s="10"/>
-      <c r="I41" s="10"/>
+      <c r="F41" s="11"/>
+      <c r="G41" s="11"/>
+      <c r="H41" s="11"/>
+      <c r="I41" s="11"/>
       <c r="J41" s="11" t="str">
         <f aca="false">IF(COUNT(F41:I41)=0,"",SUM(F41:I41))</f>
         <v/>
       </c>
-      <c r="K41" s="12" t="str">
+      <c r="K41" s="11" t="str">
         <f aca="false">IF(J41="","",IF(J41&gt;=8,"A",IF(J41&gt;=5,"B","C")))</f>
         <v/>
       </c>
       <c r="L41" s="14"/>
       <c r="M41" s="14"/>
+      <c r="N41" s="14"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="K2:K41">
@@ -2045,7 +1845,7 @@
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>"B"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>"C"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>